<commit_message>
zhengli done but not solve problem
</commit_message>
<xml_diff>
--- a/2026_09_21/LSLS/report_for_BD_template.xlsx
+++ b/2026_09_21/LSLS/report_for_BD_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lenalee\work\2026_09\2026_09_21\LSLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1DECF2C-48B5-4327-9E2D-5C4F18E7C005}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A737500-7964-428E-B785-FBF4DB3E7721}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19560" windowHeight="12405" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,21 +37,6 @@
   </si>
   <si>
     <t>App</t>
-  </si>
-  <si>
-    <r>
-      <t>少鹽少糖食店</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>SR1 page view</t>
-    </r>
   </si>
   <si>
     <t>Mobile Web</t>
@@ -83,11 +68,23 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Daily Theme Listing Impressions</t>
+      <t>Daily Brand Page (LMS) Pageview/ Impressions</t>
     </r>
   </si>
   <si>
-    <t>少鹽少糖食店 Daily Badge impression by device</t>
+    <r>
+      <t>少鹽少糖食店</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Daily Theme Listing Impressions</t>
+    </r>
   </si>
   <si>
     <r>
@@ -101,7 +98,23 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Daily Brand Page (LMS) Pageview/ Impressions</t>
+      <t>SR1 page view</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">少鹽少糖食店 </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Daily Badge impression by device</t>
     </r>
   </si>
 </sst>
@@ -109,7 +122,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -160,6 +173,14 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -587,7 +608,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -616,7 +637,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="3"/>
@@ -629,7 +650,7 @@
         <v>0</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D7" s="10" t="s">
         <v>1</v>
@@ -857,7 +878,7 @@
     </row>
     <row r="41" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A41" s="4" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
@@ -1213,7 +1234,7 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="3"/>
@@ -1226,7 +1247,7 @@
         <v>0</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D2" s="10" t="s">
         <v>1</v>
@@ -1469,199 +1490,199 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" t="s">
         <v>8</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>9</v>
-      </c>
-      <c r="C1" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="16"/>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="16"/>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="16"/>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="16"/>
       <c r="B5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="16"/>
       <c r="B6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="16"/>
       <c r="B7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="16"/>
       <c r="B8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="16"/>
       <c r="B9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="16"/>
       <c r="B10" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="16"/>
       <c r="B11" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="16"/>
       <c r="B12" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="16"/>
       <c r="B13" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="16"/>
       <c r="B14" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="16"/>
       <c r="B15" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="16"/>
       <c r="B16" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="16"/>
       <c r="B17" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="16"/>
       <c r="B18" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="16"/>
       <c r="B19" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="16"/>
       <c r="B20" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="16"/>
       <c r="B21" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="16"/>
       <c r="B22" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="16"/>
       <c r="B23" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="16"/>
       <c r="B24" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="16"/>
       <c r="B25" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="16"/>
       <c r="B26" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="16"/>
       <c r="B27" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="16"/>
       <c r="B28" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="16"/>
       <c r="B29" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="16"/>
       <c r="B30" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="16"/>
       <c r="B31" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="16"/>
       <c r="B32" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>